<commit_message>
Update Report Minus Packing
</commit_message>
<xml_diff>
--- a/Template/template_spk_planning.xlsx
+++ b/Template/template_spk_planning.xlsx
@@ -188,14 +188,14 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="28"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -203,27 +203,27 @@
       <sz val="52"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="28"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color theme="1"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -231,26 +231,26 @@
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="26"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -258,7 +258,7 @@
       <sz val="22"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -266,20 +266,20 @@
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -292,32 +292,32 @@
       <sz val="16"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="18"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -345,7 +345,7 @@
       <sz val="18"/>
       <color theme="1"/>
       <name val="Tahoma"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -750,7 +750,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="100">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -979,6 +979,9 @@
     <xf numFmtId="164" fontId="21" fillId="2" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1024,9 +1027,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1367,7 +1380,7 @@
     <col min="1" max="1" width="22" style="1" customWidth="1"/>
     <col min="2" max="2" width="42.5703125" style="1" customWidth="1"/>
     <col min="3" max="3" width="24.7109375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18" style="104" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="27.28515625" style="1" customWidth="1"/>
     <col min="6" max="6" width="29.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="23.28515625" style="1" customWidth="1"/>
@@ -1380,49 +1393,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:47" ht="57" customHeight="1">
-      <c r="A1" s="84"/>
-      <c r="B1" s="85"/>
-      <c r="C1" s="90" t="s">
+      <c r="A1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="91" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="91"/>
-      <c r="E1" s="91"/>
-      <c r="F1" s="91"/>
-      <c r="G1" s="91"/>
-      <c r="H1" s="91"/>
-      <c r="I1" s="91"/>
-      <c r="J1" s="91"/>
-      <c r="K1" s="91"/>
-      <c r="L1" s="91"/>
-      <c r="M1" s="91"/>
-      <c r="N1" s="91"/>
-      <c r="O1" s="91"/>
-      <c r="P1" s="91"/>
-      <c r="Q1" s="91"/>
-      <c r="R1" s="91"/>
-      <c r="S1" s="91"/>
-      <c r="T1" s="91"/>
-      <c r="U1" s="91"/>
-      <c r="V1" s="91"/>
-      <c r="W1" s="91"/>
-      <c r="X1" s="91"/>
-      <c r="Y1" s="91"/>
-      <c r="Z1" s="91"/>
-      <c r="AA1" s="91"/>
-      <c r="AB1" s="91"/>
-      <c r="AC1" s="91"/>
-      <c r="AD1" s="91"/>
-      <c r="AE1" s="91"/>
-      <c r="AF1" s="91"/>
-      <c r="AG1" s="91"/>
-      <c r="AH1" s="91"/>
-      <c r="AI1" s="91"/>
-      <c r="AJ1" s="91"/>
-      <c r="AK1" s="92"/>
+      <c r="D1" s="92"/>
+      <c r="E1" s="92"/>
+      <c r="F1" s="92"/>
+      <c r="G1" s="92"/>
+      <c r="H1" s="92"/>
+      <c r="I1" s="92"/>
+      <c r="J1" s="92"/>
+      <c r="K1" s="92"/>
+      <c r="L1" s="92"/>
+      <c r="M1" s="92"/>
+      <c r="N1" s="92"/>
+      <c r="O1" s="92"/>
+      <c r="P1" s="92"/>
+      <c r="Q1" s="92"/>
+      <c r="R1" s="92"/>
+      <c r="S1" s="92"/>
+      <c r="T1" s="92"/>
+      <c r="U1" s="92"/>
+      <c r="V1" s="92"/>
+      <c r="W1" s="92"/>
+      <c r="X1" s="92"/>
+      <c r="Y1" s="92"/>
+      <c r="Z1" s="92"/>
+      <c r="AA1" s="92"/>
+      <c r="AB1" s="92"/>
+      <c r="AC1" s="92"/>
+      <c r="AD1" s="92"/>
+      <c r="AE1" s="92"/>
+      <c r="AF1" s="92"/>
+      <c r="AG1" s="92"/>
+      <c r="AH1" s="92"/>
+      <c r="AI1" s="92"/>
+      <c r="AJ1" s="92"/>
+      <c r="AK1" s="93"/>
     </row>
     <row r="2" spans="1:47" ht="57" customHeight="1">
-      <c r="A2" s="86"/>
-      <c r="B2" s="87"/>
+      <c r="A2" s="87"/>
+      <c r="B2" s="88"/>
       <c r="C2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1468,8 +1481,8 @@
       <c r="AK2" s="7"/>
     </row>
     <row r="3" spans="1:47" ht="57" customHeight="1" thickBot="1">
-      <c r="A3" s="88"/>
-      <c r="B3" s="89"/>
+      <c r="A3" s="89"/>
+      <c r="B3" s="90"/>
       <c r="C3" s="8" t="s">
         <v>4</v>
       </c>
@@ -1514,8 +1527,12 @@
       <c r="AJ3" s="12"/>
       <c r="AK3" s="13"/>
     </row>
-    <row r="4" spans="1:47" ht="32.25" hidden="1" customHeight="1"/>
-    <row r="5" spans="1:47" ht="32.25" hidden="1" customHeight="1"/>
+    <row r="4" spans="1:47" ht="32.25" hidden="1" customHeight="1">
+      <c r="D4" s="1"/>
+    </row>
+    <row r="5" spans="1:47" ht="32.25" hidden="1" customHeight="1">
+      <c r="D5" s="1"/>
+    </row>
     <row r="6" spans="1:47" s="18" customFormat="1" ht="27.75" customHeight="1">
       <c r="A6" s="14" t="s">
         <v>7</v>
@@ -1526,15 +1543,15 @@
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
       <c r="G6" s="16"/>
-      <c r="H6" s="93" t="s">
+      <c r="H6" s="94" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="94"/>
-      <c r="J6" s="94"/>
-      <c r="K6" s="94"/>
-      <c r="L6" s="94"/>
-      <c r="M6" s="94"/>
-      <c r="N6" s="95"/>
+      <c r="I6" s="95"/>
+      <c r="J6" s="95"/>
+      <c r="K6" s="95"/>
+      <c r="L6" s="95"/>
+      <c r="M6" s="95"/>
+      <c r="N6" s="96"/>
       <c r="O6" s="17"/>
       <c r="Y6" s="19"/>
       <c r="Z6" s="19"/>
@@ -1572,13 +1589,13 @@
       <c r="E7" s="23"/>
       <c r="F7" s="16"/>
       <c r="G7" s="24"/>
-      <c r="H7" s="96"/>
-      <c r="I7" s="97"/>
-      <c r="J7" s="97"/>
-      <c r="K7" s="97"/>
-      <c r="L7" s="97"/>
-      <c r="M7" s="97"/>
-      <c r="N7" s="98"/>
+      <c r="H7" s="97"/>
+      <c r="I7" s="98"/>
+      <c r="J7" s="98"/>
+      <c r="K7" s="98"/>
+      <c r="L7" s="98"/>
+      <c r="M7" s="98"/>
+      <c r="N7" s="99"/>
       <c r="O7" s="25"/>
       <c r="P7" s="25"/>
       <c r="Q7" s="25"/>
@@ -1958,7 +1975,7 @@
       <c r="C13" s="50" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="51">
+      <c r="D13" s="100">
         <v>260518</v>
       </c>
       <c r="E13" s="51">
@@ -1973,22 +1990,22 @@
       <c r="H13" s="52">
         <v>507</v>
       </c>
-      <c r="I13" s="99">
+      <c r="I13" s="84">
         <v>50</v>
       </c>
-      <c r="J13" s="99">
+      <c r="J13" s="84">
         <v>50</v>
       </c>
-      <c r="K13" s="99">
+      <c r="K13" s="84">
         <v>50</v>
       </c>
-      <c r="L13" s="99">
+      <c r="L13" s="84">
         <v>50</v>
       </c>
-      <c r="M13" s="99">
+      <c r="M13" s="84">
         <v>50</v>
       </c>
-      <c r="N13" s="99">
+      <c r="N13" s="84">
         <v>50</v>
       </c>
       <c r="O13" s="62"/>
@@ -2038,7 +2055,7 @@
       <c r="C14" s="54" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="65">
+      <c r="D14" s="101">
         <v>260525</v>
       </c>
       <c r="E14" s="65">
@@ -2112,7 +2129,7 @@
       <c r="A15" s="69"/>
       <c r="B15" s="69"/>
       <c r="C15" s="69"/>
-      <c r="D15" s="70"/>
+      <c r="D15" s="102"/>
       <c r="E15" s="71"/>
       <c r="F15" s="71"/>
       <c r="G15" s="70"/>
@@ -2164,7 +2181,7 @@
       <c r="A16" s="69"/>
       <c r="B16" s="69"/>
       <c r="C16" s="69"/>
-      <c r="D16" s="70"/>
+      <c r="D16" s="102"/>
       <c r="E16" s="71"/>
       <c r="F16" s="71"/>
       <c r="G16" s="70"/>
@@ -2216,7 +2233,7 @@
       <c r="A17" s="69"/>
       <c r="B17" s="69"/>
       <c r="C17" s="69"/>
-      <c r="D17" s="70"/>
+      <c r="D17" s="102"/>
       <c r="E17" s="71"/>
       <c r="F17" s="71"/>
       <c r="G17" s="70"/>
@@ -2268,7 +2285,7 @@
       <c r="A18" s="69"/>
       <c r="B18" s="69"/>
       <c r="C18" s="69"/>
-      <c r="D18" s="70"/>
+      <c r="D18" s="102"/>
       <c r="E18" s="71"/>
       <c r="F18" s="71"/>
       <c r="G18" s="70"/>
@@ -2320,7 +2337,7 @@
       <c r="A19" s="69"/>
       <c r="B19" s="69"/>
       <c r="C19" s="69"/>
-      <c r="D19" s="70"/>
+      <c r="D19" s="102"/>
       <c r="E19" s="71"/>
       <c r="F19" s="71"/>
       <c r="G19" s="70"/>
@@ -2372,7 +2389,7 @@
       <c r="A20" s="69"/>
       <c r="B20" s="69"/>
       <c r="C20" s="69"/>
-      <c r="D20" s="70"/>
+      <c r="D20" s="102"/>
       <c r="E20" s="71"/>
       <c r="F20" s="71"/>
       <c r="G20" s="70"/>
@@ -2424,7 +2441,7 @@
       <c r="A21" s="69"/>
       <c r="B21" s="69"/>
       <c r="C21" s="69"/>
-      <c r="D21" s="70"/>
+      <c r="D21" s="102"/>
       <c r="E21" s="71"/>
       <c r="F21" s="71"/>
       <c r="G21" s="70"/>
@@ -2476,7 +2493,7 @@
       <c r="A22" s="69"/>
       <c r="B22" s="69"/>
       <c r="C22" s="69"/>
-      <c r="D22" s="70"/>
+      <c r="D22" s="102"/>
       <c r="E22" s="71"/>
       <c r="F22" s="71"/>
       <c r="G22" s="70"/>
@@ -2528,7 +2545,7 @@
       <c r="A23" s="69"/>
       <c r="B23" s="69"/>
       <c r="C23" s="69"/>
-      <c r="D23" s="70"/>
+      <c r="D23" s="102"/>
       <c r="E23" s="71"/>
       <c r="F23" s="71"/>
       <c r="G23" s="70"/>
@@ -2580,7 +2597,7 @@
       <c r="A24" s="74"/>
       <c r="B24" s="69"/>
       <c r="C24" s="69"/>
-      <c r="D24" s="70"/>
+      <c r="D24" s="102"/>
       <c r="E24" s="75"/>
       <c r="F24" s="75"/>
       <c r="G24" s="76"/>
@@ -2632,7 +2649,7 @@
       <c r="A25" s="74"/>
       <c r="B25" s="69"/>
       <c r="C25" s="69"/>
-      <c r="D25" s="70"/>
+      <c r="D25" s="102"/>
       <c r="E25" s="75"/>
       <c r="F25" s="75"/>
       <c r="G25" s="76"/>
@@ -2684,7 +2701,7 @@
       <c r="A26" s="74"/>
       <c r="B26" s="69"/>
       <c r="C26" s="69"/>
-      <c r="D26" s="70"/>
+      <c r="D26" s="102"/>
       <c r="E26" s="75"/>
       <c r="F26" s="75"/>
       <c r="G26" s="76"/>
@@ -2736,7 +2753,7 @@
       <c r="A27" s="74"/>
       <c r="B27" s="69"/>
       <c r="C27" s="69"/>
-      <c r="D27" s="70"/>
+      <c r="D27" s="102"/>
       <c r="E27" s="75"/>
       <c r="F27" s="75"/>
       <c r="G27" s="76"/>
@@ -2788,7 +2805,7 @@
       <c r="A28" s="74"/>
       <c r="B28" s="69"/>
       <c r="C28" s="69"/>
-      <c r="D28" s="70"/>
+      <c r="D28" s="102"/>
       <c r="E28" s="75"/>
       <c r="F28" s="75"/>
       <c r="G28" s="76"/>
@@ -2840,7 +2857,7 @@
       <c r="A29" s="74"/>
       <c r="B29" s="69"/>
       <c r="C29" s="69"/>
-      <c r="D29" s="70"/>
+      <c r="D29" s="102"/>
       <c r="E29" s="75"/>
       <c r="F29" s="75"/>
       <c r="G29" s="76"/>
@@ -2892,7 +2909,7 @@
       <c r="A30" s="74"/>
       <c r="B30" s="69"/>
       <c r="C30" s="69"/>
-      <c r="D30" s="70"/>
+      <c r="D30" s="102"/>
       <c r="E30" s="75"/>
       <c r="F30" s="75"/>
       <c r="G30" s="76"/>
@@ -2944,7 +2961,7 @@
       <c r="A31" s="74"/>
       <c r="B31" s="69"/>
       <c r="C31" s="69"/>
-      <c r="D31" s="70"/>
+      <c r="D31" s="102"/>
       <c r="E31" s="75"/>
       <c r="F31" s="75"/>
       <c r="G31" s="76"/>
@@ -2996,7 +3013,7 @@
       <c r="A32" s="74"/>
       <c r="B32" s="69"/>
       <c r="C32" s="69"/>
-      <c r="D32" s="70"/>
+      <c r="D32" s="102"/>
       <c r="E32" s="75"/>
       <c r="F32" s="75"/>
       <c r="G32" s="76"/>
@@ -3048,7 +3065,7 @@
       <c r="A33" s="74"/>
       <c r="B33" s="69"/>
       <c r="C33" s="69"/>
-      <c r="D33" s="70"/>
+      <c r="D33" s="102"/>
       <c r="E33" s="75"/>
       <c r="F33" s="75"/>
       <c r="G33" s="76"/>
@@ -3100,7 +3117,7 @@
       <c r="A34" s="74"/>
       <c r="B34" s="69"/>
       <c r="C34" s="69"/>
-      <c r="D34" s="70"/>
+      <c r="D34" s="102"/>
       <c r="E34" s="75"/>
       <c r="F34" s="75"/>
       <c r="G34" s="76"/>
@@ -3152,7 +3169,7 @@
       <c r="A35" s="74"/>
       <c r="B35" s="69"/>
       <c r="C35" s="69"/>
-      <c r="D35" s="70"/>
+      <c r="D35" s="102"/>
       <c r="E35" s="75"/>
       <c r="F35" s="75"/>
       <c r="G35" s="76"/>
@@ -3204,7 +3221,7 @@
       <c r="A36" s="74"/>
       <c r="B36" s="69"/>
       <c r="C36" s="69"/>
-      <c r="D36" s="70"/>
+      <c r="D36" s="102"/>
       <c r="E36" s="75"/>
       <c r="F36" s="75"/>
       <c r="G36" s="76"/>
@@ -3256,7 +3273,7 @@
       <c r="A37" s="74"/>
       <c r="B37" s="69"/>
       <c r="C37" s="69"/>
-      <c r="D37" s="70"/>
+      <c r="D37" s="102"/>
       <c r="E37" s="75"/>
       <c r="F37" s="75"/>
       <c r="G37" s="76"/>
@@ -3308,7 +3325,7 @@
       <c r="A38" s="74"/>
       <c r="B38" s="69"/>
       <c r="C38" s="69"/>
-      <c r="D38" s="70"/>
+      <c r="D38" s="102"/>
       <c r="E38" s="75"/>
       <c r="F38" s="75"/>
       <c r="G38" s="76"/>
@@ -3360,7 +3377,7 @@
       <c r="A39" s="74"/>
       <c r="B39" s="69"/>
       <c r="C39" s="69"/>
-      <c r="D39" s="70"/>
+      <c r="D39" s="102"/>
       <c r="E39" s="75"/>
       <c r="F39" s="75"/>
       <c r="G39" s="76"/>
@@ -3412,7 +3429,7 @@
       <c r="A40" s="74"/>
       <c r="B40" s="69"/>
       <c r="C40" s="69"/>
-      <c r="D40" s="70"/>
+      <c r="D40" s="102"/>
       <c r="E40" s="75"/>
       <c r="F40" s="75"/>
       <c r="G40" s="76"/>
@@ -3464,7 +3481,7 @@
       <c r="A41" s="78"/>
       <c r="B41" s="69"/>
       <c r="C41" s="69"/>
-      <c r="D41" s="70"/>
+      <c r="D41" s="102"/>
       <c r="E41" s="75"/>
       <c r="F41" s="75"/>
       <c r="G41" s="76"/>
@@ -3516,7 +3533,7 @@
       <c r="A42" s="78"/>
       <c r="B42" s="69"/>
       <c r="C42" s="78"/>
-      <c r="D42" s="76"/>
+      <c r="D42" s="103"/>
       <c r="E42" s="75"/>
       <c r="F42" s="75"/>
       <c r="G42" s="76"/>
@@ -3568,7 +3585,7 @@
       <c r="A43" s="74"/>
       <c r="B43" s="69"/>
       <c r="C43" s="74"/>
-      <c r="D43" s="76"/>
+      <c r="D43" s="103"/>
       <c r="E43" s="75"/>
       <c r="F43" s="75"/>
       <c r="G43" s="76"/>
@@ -3620,7 +3637,7 @@
       <c r="A44" s="74"/>
       <c r="B44" s="69"/>
       <c r="C44" s="74"/>
-      <c r="D44" s="76"/>
+      <c r="D44" s="103"/>
       <c r="E44" s="75"/>
       <c r="F44" s="75"/>
       <c r="G44" s="76"/>
@@ -3672,7 +3689,7 @@
       <c r="A45" s="74"/>
       <c r="B45" s="69"/>
       <c r="C45" s="74"/>
-      <c r="D45" s="76"/>
+      <c r="D45" s="103"/>
       <c r="E45" s="75"/>
       <c r="F45" s="75"/>
       <c r="G45" s="76"/>
@@ -3724,7 +3741,7 @@
       <c r="A46" s="74"/>
       <c r="B46" s="69"/>
       <c r="C46" s="74"/>
-      <c r="D46" s="76"/>
+      <c r="D46" s="103"/>
       <c r="E46" s="75"/>
       <c r="F46" s="69"/>
       <c r="G46" s="76"/>
@@ -3776,7 +3793,7 @@
       <c r="A47" s="74"/>
       <c r="B47" s="69"/>
       <c r="C47" s="74"/>
-      <c r="D47" s="76"/>
+      <c r="D47" s="103"/>
       <c r="E47" s="75"/>
       <c r="F47" s="69"/>
       <c r="G47" s="76"/>
@@ -3828,7 +3845,7 @@
       <c r="A48" s="74"/>
       <c r="B48" s="69"/>
       <c r="C48" s="74"/>
-      <c r="D48" s="76"/>
+      <c r="D48" s="103"/>
       <c r="E48" s="75"/>
       <c r="F48" s="69"/>
       <c r="G48" s="76"/>
@@ -3880,7 +3897,7 @@
       <c r="A49" s="78"/>
       <c r="B49" s="69"/>
       <c r="C49" s="74"/>
-      <c r="D49" s="76"/>
+      <c r="D49" s="103"/>
       <c r="E49" s="75"/>
       <c r="F49" s="75"/>
       <c r="G49" s="76"/>
@@ -3932,7 +3949,7 @@
       <c r="A50" s="78"/>
       <c r="B50" s="69"/>
       <c r="C50" s="74"/>
-      <c r="D50" s="76"/>
+      <c r="D50" s="103"/>
       <c r="E50" s="75"/>
       <c r="F50" s="75"/>
       <c r="G50" s="76"/>

</xml_diff>